<commit_message>
Update packaged data workbooks
</commit_message>
<xml_diff>
--- a/src/moodys_datahub/data/data_dict_available.xlsx
+++ b/src/moodys_datahub/data/data_dict_available.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://studentcbs-my.sharepoint.com/personal/kgp_libas_cbs_dk/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://studentcbs-my.sharepoint.com/personal/kgp_libas_cbs_dk/Documents/Desktop/moody-s_datahub/src/moodys_datahub/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="97" documentId="13_ncr:1_{1AD8FFE2-977B-4D40-9991-3401343FE025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9FA1F74-5CD3-46F3-92AA-B905FC8EE67E}"/>
+  <xr:revisionPtr revIDLastSave="108" documentId="13_ncr:1_{1AD8FFE2-977B-4D40-9991-3401343FE025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12A61353-5236-414A-A454-9F87DEACA1EC}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6563,6 +6563,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -6638,7 +6639,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -6656,10 +6657,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Update available data dictionary workbook
</commit_message>
<xml_diff>
--- a/src/moodys_datahub/data/data_dict_available.xlsx
+++ b/src/moodys_datahub/data/data_dict_available.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://studentcbs-my.sharepoint.com/personal/kgp_libas_cbs_dk/Documents/Desktop/moody-s_datahub/src/moodys_datahub/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="137" documentId="13_ncr:1_{1AD8FFE2-977B-4D40-9991-3401343FE025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6FAABDFC-3B8A-4292-8E0B-A1824916F4E5}"/>
+  <xr:revisionPtr revIDLastSave="143" documentId="13_ncr:1_{1AD8FFE2-977B-4D40-9991-3401343FE025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B36E7DC5-7F63-4744-8738-FD03DB5DF742}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="-27330" yWindow="5055" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -6963,7 +6963,7 @@
     <col min="2" max="2" width="63.42578125" customWidth="1"/>
     <col min="3" max="3" width="55" customWidth="1"/>
     <col min="4" max="4" width="45" customWidth="1"/>
-    <col min="5" max="5" width="46.28515625" customWidth="1"/>
+    <col min="5" max="5" width="112.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7763,7 +7763,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -7774,10 +7774,10 @@
         <v>2088</v>
       </c>
       <c r="D41" t="s">
-        <v>313</v>
+        <v>464</v>
       </c>
       <c r="E41" t="s">
-        <v>356</v>
+        <v>465</v>
       </c>
       <c r="F41" t="s">
         <v>2112</v>
@@ -8788,16 +8788,16 @@
         <v>91</v>
       </c>
       <c r="B92" t="s">
-        <v>2011</v>
+        <v>2087</v>
       </c>
       <c r="C92" t="s">
-        <v>2088</v>
+        <v>333</v>
       </c>
       <c r="D92" t="s">
-        <v>456</v>
+        <v>464</v>
       </c>
       <c r="E92" t="s">
-        <v>457</v>
+        <v>465</v>
       </c>
       <c r="F92" t="s">
         <v>2112</v>
@@ -8868,10 +8868,10 @@
         <v>95</v>
       </c>
       <c r="B96" t="s">
-        <v>2011</v>
+        <v>2091</v>
       </c>
       <c r="C96" t="s">
-        <v>2088</v>
+        <v>2092</v>
       </c>
       <c r="D96" t="s">
         <v>464</v>
@@ -9468,16 +9468,16 @@
         <v>125</v>
       </c>
       <c r="B126" t="s">
-        <v>2011</v>
+        <v>2016</v>
       </c>
       <c r="C126" t="s">
-        <v>2088</v>
+        <v>994</v>
       </c>
       <c r="D126" t="s">
-        <v>519</v>
+        <v>464</v>
       </c>
       <c r="E126" t="s">
-        <v>520</v>
+        <v>465</v>
       </c>
       <c r="F126" t="s">
         <v>2112</v>
@@ -10023,7 +10023,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" s="1">
         <v>153</v>
       </c>
@@ -10031,13 +10031,13 @@
         <v>2011</v>
       </c>
       <c r="C154" t="s">
-        <v>2089</v>
+        <v>2088</v>
       </c>
       <c r="D154" t="s">
-        <v>313</v>
+        <v>456</v>
       </c>
       <c r="E154" t="s">
-        <v>314</v>
+        <v>457</v>
       </c>
       <c r="F154" t="s">
         <v>2112</v>
@@ -11508,16 +11508,16 @@
         <v>227</v>
       </c>
       <c r="B228" t="s">
-        <v>2011</v>
+        <v>2087</v>
       </c>
       <c r="C228" t="s">
-        <v>2089</v>
+        <v>333</v>
       </c>
       <c r="D228" t="s">
-        <v>664</v>
+        <v>456</v>
       </c>
       <c r="E228" t="s">
-        <v>665</v>
+        <v>457</v>
       </c>
       <c r="F228" t="s">
         <v>2112</v>
@@ -11863,21 +11863,21 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A246" s="1">
         <v>245</v>
       </c>
       <c r="B246" t="s">
-        <v>2011</v>
+        <v>2091</v>
       </c>
       <c r="C246" t="s">
-        <v>2090</v>
+        <v>2092</v>
       </c>
       <c r="D246" t="s">
-        <v>313</v>
+        <v>456</v>
       </c>
       <c r="E246" t="s">
-        <v>678</v>
+        <v>457</v>
       </c>
       <c r="F246" t="s">
         <v>2112</v>
@@ -12943,21 +12943,21 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="300" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A300" s="1">
         <v>299</v>
       </c>
       <c r="B300" t="s">
-        <v>2087</v>
+        <v>2016</v>
       </c>
       <c r="C300" t="s">
-        <v>333</v>
+        <v>994</v>
       </c>
       <c r="D300" t="s">
-        <v>313</v>
+        <v>456</v>
       </c>
       <c r="E300" t="s">
-        <v>356</v>
+        <v>457</v>
       </c>
       <c r="F300" t="s">
         <v>2112</v>
@@ -13968,16 +13968,16 @@
         <v>350</v>
       </c>
       <c r="B351" t="s">
-        <v>2087</v>
+        <v>2021</v>
       </c>
       <c r="C351" t="s">
-        <v>333</v>
+        <v>1591</v>
       </c>
       <c r="D351" t="s">
-        <v>456</v>
+        <v>1639</v>
       </c>
       <c r="E351" t="s">
-        <v>457</v>
+        <v>1640</v>
       </c>
       <c r="F351" t="s">
         <v>2112</v>
@@ -14048,16 +14048,16 @@
         <v>354</v>
       </c>
       <c r="B355" t="s">
-        <v>2087</v>
+        <v>2011</v>
       </c>
       <c r="C355" t="s">
-        <v>333</v>
+        <v>2088</v>
       </c>
       <c r="D355" t="s">
-        <v>464</v>
+        <v>519</v>
       </c>
       <c r="E355" t="s">
-        <v>465</v>
+        <v>520</v>
       </c>
       <c r="F355" t="s">
         <v>2112</v>
@@ -15203,21 +15203,21 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="413" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A413" s="1">
         <v>412</v>
       </c>
       <c r="B413" t="s">
-        <v>2087</v>
+        <v>2091</v>
       </c>
       <c r="C413" t="s">
-        <v>530</v>
+        <v>2092</v>
       </c>
       <c r="D413" t="s">
-        <v>313</v>
+        <v>519</v>
       </c>
       <c r="E413" t="s">
-        <v>314</v>
+        <v>520</v>
       </c>
       <c r="F413" t="s">
         <v>2112</v>
@@ -16688,16 +16688,16 @@
         <v>486</v>
       </c>
       <c r="B487" t="s">
-        <v>2087</v>
+        <v>2016</v>
       </c>
       <c r="C487" t="s">
-        <v>530</v>
+        <v>994</v>
       </c>
       <c r="D487" t="s">
-        <v>664</v>
+        <v>519</v>
       </c>
       <c r="E487" t="s">
-        <v>665</v>
+        <v>520</v>
       </c>
       <c r="F487" t="s">
         <v>2112</v>
@@ -17043,21 +17043,21 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="505" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="505" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A505" s="1">
         <v>504</v>
       </c>
       <c r="B505" t="s">
-        <v>2087</v>
+        <v>2011</v>
       </c>
       <c r="C505" t="s">
-        <v>670</v>
+        <v>2088</v>
       </c>
       <c r="D505" t="s">
         <v>313</v>
       </c>
       <c r="E505" t="s">
-        <v>678</v>
+        <v>356</v>
       </c>
       <c r="F505" t="s">
         <v>2112</v>
@@ -17723,7 +17723,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="539" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="539" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A539" s="1">
         <v>538</v>
       </c>
@@ -17743,7 +17743,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="540" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="540" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A540" s="1">
         <v>539</v>
       </c>
@@ -17763,7 +17763,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="541" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="541" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A541" s="1">
         <v>540</v>
       </c>
@@ -17783,7 +17783,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="542" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="542" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A542" s="1">
         <v>541</v>
       </c>
@@ -17803,7 +17803,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="543" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="543" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A543" s="1">
         <v>542</v>
       </c>
@@ -17823,7 +17823,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="544" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="544" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A544" s="1">
         <v>543</v>
       </c>
@@ -17843,7 +17843,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="545" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="545" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A545" s="1">
         <v>544</v>
       </c>
@@ -17863,7 +17863,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="546" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="546" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A546" s="1">
         <v>545</v>
       </c>
@@ -17883,7 +17883,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="547" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="547" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A547" s="1">
         <v>546</v>
       </c>
@@ -17903,7 +17903,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="548" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="548" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A548" s="1">
         <v>547</v>
       </c>
@@ -17923,7 +17923,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="549" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="549" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A549" s="1">
         <v>548</v>
       </c>
@@ -17943,7 +17943,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="550" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="550" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A550" s="1">
         <v>549</v>
       </c>
@@ -17963,7 +17963,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="551" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="551" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A551" s="1">
         <v>550</v>
       </c>
@@ -17983,7 +17983,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="552" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="552" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A552" s="1">
         <v>551</v>
       </c>
@@ -18003,7 +18003,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="553" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="553" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A553" s="1">
         <v>552</v>
       </c>
@@ -18023,7 +18023,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="554" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="554" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A554" s="1">
         <v>553</v>
       </c>
@@ -18043,7 +18043,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="555" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="555" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A555" s="1">
         <v>554</v>
       </c>
@@ -18063,7 +18063,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="556" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="556" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A556" s="1">
         <v>555</v>
       </c>
@@ -18083,7 +18083,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="557" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="557" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A557" s="1">
         <v>556</v>
       </c>
@@ -18103,7 +18103,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="558" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="558" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A558" s="1">
         <v>557</v>
       </c>
@@ -18123,7 +18123,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="559" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="559" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A559" s="1">
         <v>558</v>
       </c>
@@ -18143,7 +18143,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="560" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="560" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A560" s="1">
         <v>559</v>
       </c>
@@ -18163,7 +18163,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="561" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="561" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A561" s="1">
         <v>560</v>
       </c>
@@ -18183,7 +18183,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="562" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="562" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A562" s="1">
         <v>561</v>
       </c>
@@ -18203,7 +18203,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="563" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="563" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A563" s="1">
         <v>562</v>
       </c>
@@ -18223,7 +18223,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="564" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="564" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A564" s="1">
         <v>563</v>
       </c>
@@ -18243,7 +18243,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="565" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="565" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A565" s="1">
         <v>564</v>
       </c>
@@ -18263,7 +18263,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="566" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="566" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A566" s="1">
         <v>565</v>
       </c>
@@ -18283,7 +18283,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="567" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="567" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A567" s="1">
         <v>566</v>
       </c>
@@ -18303,7 +18303,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="568" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="568" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A568" s="1">
         <v>567</v>
       </c>
@@ -18323,7 +18323,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="569" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="569" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A569" s="1">
         <v>568</v>
       </c>
@@ -18343,7 +18343,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="570" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="570" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A570" s="1">
         <v>569</v>
       </c>
@@ -18363,7 +18363,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="571" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="571" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A571" s="1">
         <v>570</v>
       </c>
@@ -18383,7 +18383,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="572" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="572" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A572" s="1">
         <v>571</v>
       </c>
@@ -18403,7 +18403,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="573" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="573" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A573" s="1">
         <v>572</v>
       </c>
@@ -18423,7 +18423,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="574" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="574" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A574" s="1">
         <v>573</v>
       </c>
@@ -18443,7 +18443,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="575" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="575" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A575" s="1">
         <v>574</v>
       </c>
@@ -18463,7 +18463,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="576" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="576" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A576" s="1">
         <v>575</v>
       </c>
@@ -18483,7 +18483,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="577" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="577" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A577" s="1">
         <v>576</v>
       </c>
@@ -18503,7 +18503,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="578" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="578" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A578" s="1">
         <v>577</v>
       </c>
@@ -18523,7 +18523,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="579" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="579" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A579" s="1">
         <v>578</v>
       </c>
@@ -18543,7 +18543,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="580" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="580" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A580" s="1">
         <v>579</v>
       </c>
@@ -18563,7 +18563,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="581" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="581" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A581" s="1">
         <v>580</v>
       </c>
@@ -18583,7 +18583,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="582" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="582" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A582" s="1">
         <v>581</v>
       </c>
@@ -19003,21 +19003,21 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="603" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="603" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A603" s="1">
         <v>602</v>
       </c>
       <c r="B603" t="s">
-        <v>2091</v>
+        <v>2011</v>
       </c>
       <c r="C603" t="s">
-        <v>2092</v>
+        <v>2089</v>
       </c>
       <c r="D603" t="s">
         <v>313</v>
       </c>
       <c r="E603" t="s">
-        <v>356</v>
+        <v>314</v>
       </c>
       <c r="F603" t="s">
         <v>2112</v>
@@ -20028,16 +20028,16 @@
         <v>653</v>
       </c>
       <c r="B654" t="s">
-        <v>2091</v>
+        <v>2011</v>
       </c>
       <c r="C654" t="s">
-        <v>2092</v>
+        <v>2090</v>
       </c>
       <c r="D654" t="s">
-        <v>456</v>
+        <v>313</v>
       </c>
       <c r="E654" t="s">
-        <v>457</v>
+        <v>678</v>
       </c>
       <c r="F654" t="s">
         <v>2112</v>
@@ -20108,16 +20108,16 @@
         <v>657</v>
       </c>
       <c r="B658" t="s">
-        <v>2091</v>
+        <v>2087</v>
       </c>
       <c r="C658" t="s">
-        <v>2092</v>
+        <v>333</v>
       </c>
       <c r="D658" t="s">
-        <v>464</v>
+        <v>313</v>
       </c>
       <c r="E658" t="s">
-        <v>465</v>
+        <v>356</v>
       </c>
       <c r="F658" t="s">
         <v>2112</v>
@@ -20708,16 +20708,16 @@
         <v>687</v>
       </c>
       <c r="B688" t="s">
-        <v>2091</v>
+        <v>2087</v>
       </c>
       <c r="C688" t="s">
-        <v>2092</v>
+        <v>530</v>
       </c>
       <c r="D688" t="s">
-        <v>519</v>
+        <v>313</v>
       </c>
       <c r="E688" t="s">
-        <v>520</v>
+        <v>314</v>
       </c>
       <c r="F688" t="s">
         <v>2112</v>
@@ -21263,21 +21263,21 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="716" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="716" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A716" s="1">
         <v>715</v>
       </c>
       <c r="B716" t="s">
-        <v>2091</v>
+        <v>2087</v>
       </c>
       <c r="C716" t="s">
-        <v>2093</v>
+        <v>670</v>
       </c>
       <c r="D716" t="s">
         <v>313</v>
       </c>
       <c r="E716" t="s">
-        <v>314</v>
+        <v>678</v>
       </c>
       <c r="F716" t="s">
         <v>2112</v>
@@ -22751,13 +22751,13 @@
         <v>2091</v>
       </c>
       <c r="C790" t="s">
-        <v>2093</v>
+        <v>2092</v>
       </c>
       <c r="D790" t="s">
-        <v>664</v>
+        <v>313</v>
       </c>
       <c r="E790" t="s">
-        <v>665</v>
+        <v>356</v>
       </c>
       <c r="F790" t="s">
         <v>2112</v>
@@ -23103,7 +23103,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="808" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="808" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A808" s="1">
         <v>807</v>
       </c>
@@ -23111,13 +23111,13 @@
         <v>2091</v>
       </c>
       <c r="C808" t="s">
-        <v>2094</v>
+        <v>2093</v>
       </c>
       <c r="D808" t="s">
         <v>313</v>
       </c>
       <c r="E808" t="s">
-        <v>678</v>
+        <v>314</v>
       </c>
       <c r="F808" t="s">
         <v>2112</v>
@@ -24083,7 +24083,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="857" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="857" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A857" s="1">
         <v>856</v>
       </c>
@@ -24091,13 +24091,13 @@
         <v>2091</v>
       </c>
       <c r="C857" t="s">
-        <v>2099</v>
+        <v>2094</v>
       </c>
       <c r="D857" t="s">
         <v>313</v>
       </c>
       <c r="E857" t="s">
-        <v>314</v>
+        <v>678</v>
       </c>
       <c r="F857" t="s">
         <v>2112</v>
@@ -24583,7 +24583,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="882" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="882" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A882" s="1">
         <v>881</v>
       </c>
@@ -24591,7 +24591,7 @@
         <v>2091</v>
       </c>
       <c r="C882" t="s">
-        <v>2100</v>
+        <v>2099</v>
       </c>
       <c r="D882" t="s">
         <v>313</v>
@@ -25083,7 +25083,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="907" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="907" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A907" s="1">
         <v>906</v>
       </c>
@@ -25091,13 +25091,13 @@
         <v>2091</v>
       </c>
       <c r="C907" t="s">
-        <v>2101</v>
+        <v>2100</v>
       </c>
       <c r="D907" t="s">
         <v>313</v>
       </c>
       <c r="E907" t="s">
-        <v>678</v>
+        <v>314</v>
       </c>
       <c r="F907" t="s">
         <v>2112</v>
@@ -32003,21 +32003,21 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1253" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1253" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A1253" s="1">
         <v>1252</v>
       </c>
       <c r="B1253" t="s">
-        <v>2016</v>
+        <v>2091</v>
       </c>
       <c r="C1253" t="s">
-        <v>994</v>
+        <v>2101</v>
       </c>
       <c r="D1253" t="s">
         <v>313</v>
       </c>
       <c r="E1253" t="s">
-        <v>356</v>
+        <v>678</v>
       </c>
       <c r="F1253" t="s">
         <v>2112</v>
@@ -33034,10 +33034,10 @@
         <v>994</v>
       </c>
       <c r="D1304" t="s">
-        <v>456</v>
+        <v>313</v>
       </c>
       <c r="E1304" t="s">
-        <v>457</v>
+        <v>356</v>
       </c>
       <c r="F1304" t="s">
         <v>2112</v>
@@ -33111,13 +33111,13 @@
         <v>2016</v>
       </c>
       <c r="C1308" t="s">
-        <v>994</v>
+        <v>1108</v>
       </c>
       <c r="D1308" t="s">
-        <v>464</v>
+        <v>313</v>
       </c>
       <c r="E1308" t="s">
-        <v>465</v>
+        <v>678</v>
       </c>
       <c r="F1308" t="s">
         <v>2112</v>
@@ -33708,16 +33708,16 @@
         <v>1337</v>
       </c>
       <c r="B1338" t="s">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="C1338" t="s">
-        <v>994</v>
+        <v>2107</v>
       </c>
       <c r="D1338" t="s">
-        <v>519</v>
+        <v>313</v>
       </c>
       <c r="E1338" t="s">
-        <v>520</v>
+        <v>314</v>
       </c>
       <c r="F1338" t="s">
         <v>2112</v>
@@ -37643,20 +37643,20 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1535" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1535" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A1535" s="1">
         <v>1534</v>
       </c>
       <c r="B1535" t="s">
-        <v>2016</v>
+        <v>2019</v>
       </c>
       <c r="C1535" t="s">
-        <v>1108</v>
-      </c>
-      <c r="D1535" t="s">
+        <v>847</v>
+      </c>
+      <c r="D1535" s="4" t="s">
         <v>313</v>
       </c>
-      <c r="E1535" t="s">
+      <c r="E1535" s="4" t="s">
         <v>678</v>
       </c>
       <c r="F1535" t="s">
@@ -39403,21 +39403,21 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1623" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1623" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A1623" s="1">
         <v>1622</v>
       </c>
       <c r="B1623" t="s">
-        <v>2017</v>
+        <v>2011</v>
       </c>
       <c r="C1623" t="s">
-        <v>2107</v>
+        <v>2089</v>
       </c>
       <c r="D1623" t="s">
-        <v>313</v>
+        <v>664</v>
       </c>
       <c r="E1623" t="s">
-        <v>314</v>
+        <v>665</v>
       </c>
       <c r="F1623" t="s">
         <v>2112</v>
@@ -39603,7 +39603,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1633" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1633" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1633" s="1">
         <v>1632</v>
       </c>
@@ -39623,7 +39623,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1634" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1634" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1634" s="1">
         <v>1633</v>
       </c>
@@ -39643,7 +39643,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1635" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1635" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1635" s="1">
         <v>1634</v>
       </c>
@@ -39663,7 +39663,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1636" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1636" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1636" s="1">
         <v>1635</v>
       </c>
@@ -39683,7 +39683,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1637" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1637" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1637" s="1">
         <v>1636</v>
       </c>
@@ -39703,7 +39703,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1638" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1638" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1638" s="1">
         <v>1637</v>
       </c>
@@ -39723,7 +39723,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1639" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1639" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1639" s="1">
         <v>1638</v>
       </c>
@@ -39743,7 +39743,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1640" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1640" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1640" s="1">
         <v>1639</v>
       </c>
@@ -39763,7 +39763,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1641" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1641" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1641" s="1">
         <v>1640</v>
       </c>
@@ -39783,7 +39783,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1642" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1642" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1642" s="1">
         <v>1641</v>
       </c>
@@ -39803,7 +39803,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1643" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1643" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1643" s="1">
         <v>1642</v>
       </c>
@@ -39823,7 +39823,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1644" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1644" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1644" s="1">
         <v>1643</v>
       </c>
@@ -39843,7 +39843,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1645" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1645" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1645" s="1">
         <v>1644</v>
       </c>
@@ -39863,7 +39863,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1646" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1646" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1646" s="1">
         <v>1645</v>
       </c>
@@ -39883,7 +39883,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1647" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1647" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1647" s="1">
         <v>1646</v>
       </c>
@@ -39903,7 +39903,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1648" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1648" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1648" s="1">
         <v>1647</v>
       </c>
@@ -39923,7 +39923,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1649" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1649" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1649" s="1">
         <v>1648</v>
       </c>
@@ -39943,7 +39943,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1650" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1650" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1650" s="1">
         <v>1649</v>
       </c>
@@ -39963,7 +39963,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1651" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1651" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1651" s="1">
         <v>1650</v>
       </c>
@@ -39983,7 +39983,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1652" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1652" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1652" s="1">
         <v>1651</v>
       </c>
@@ -40003,7 +40003,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1653" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1653" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1653" s="1">
         <v>1652</v>
       </c>
@@ -40023,7 +40023,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1654" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1654" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1654" s="1">
         <v>1653</v>
       </c>
@@ -40043,7 +40043,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1655" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1655" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1655" s="1">
         <v>1654</v>
       </c>
@@ -40063,7 +40063,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1656" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1656" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1656" s="1">
         <v>1655</v>
       </c>
@@ -40083,7 +40083,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1657" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1657" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1657" s="1">
         <v>1656</v>
       </c>
@@ -40103,7 +40103,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1658" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1658" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1658" s="1">
         <v>1657</v>
       </c>
@@ -40123,7 +40123,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1659" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1659" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1659" s="1">
         <v>1658</v>
       </c>
@@ -40143,7 +40143,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1660" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1660" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1660" s="1">
         <v>1659</v>
       </c>
@@ -40163,7 +40163,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1661" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1661" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1661" s="1">
         <v>1660</v>
       </c>
@@ -40183,7 +40183,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1662" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1662" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1662" s="1">
         <v>1661</v>
       </c>
@@ -40203,7 +40203,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1663" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1663" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1663" s="1">
         <v>1662</v>
       </c>
@@ -40223,7 +40223,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1664" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1664" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1664" s="1">
         <v>1663</v>
       </c>
@@ -40243,7 +40243,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1665" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1665" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1665" s="1">
         <v>1664</v>
       </c>
@@ -40263,7 +40263,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1666" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1666" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1666" s="1">
         <v>1665</v>
       </c>
@@ -40283,7 +40283,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1667" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1667" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1667" s="1">
         <v>1666</v>
       </c>
@@ -40303,7 +40303,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1668" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1668" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1668" s="1">
         <v>1667</v>
       </c>
@@ -40323,7 +40323,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1669" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1669" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1669" s="1">
         <v>1668</v>
       </c>
@@ -40343,7 +40343,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1670" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1670" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1670" s="1">
         <v>1669</v>
       </c>
@@ -40363,7 +40363,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1671" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1671" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1671" s="1">
         <v>1670</v>
       </c>
@@ -40383,7 +40383,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1672" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1672" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1672" s="1">
         <v>1671</v>
       </c>
@@ -40403,7 +40403,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1673" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1673" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1673" s="1">
         <v>1672</v>
       </c>
@@ -40423,7 +40423,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1674" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1674" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1674" s="1">
         <v>1673</v>
       </c>
@@ -40443,7 +40443,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1675" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1675" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1675" s="1">
         <v>1674</v>
       </c>
@@ -40463,7 +40463,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1676" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1676" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1676" s="1">
         <v>1675</v>
       </c>
@@ -40483,7 +40483,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1677" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1677" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1677" s="1">
         <v>1676</v>
       </c>
@@ -40503,7 +40503,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1678" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1678" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1678" s="1">
         <v>1677</v>
       </c>
@@ -40523,7 +40523,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1679" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1679" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1679" s="1">
         <v>1678</v>
       </c>
@@ -40543,7 +40543,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1680" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1680" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1680" s="1">
         <v>1679</v>
       </c>
@@ -40563,7 +40563,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1681" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1681" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1681" s="1">
         <v>1680</v>
       </c>
@@ -40583,7 +40583,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1682" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1682" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1682" s="1">
         <v>1681</v>
       </c>
@@ -40603,7 +40603,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1683" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1683" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1683" s="1">
         <v>1682</v>
       </c>
@@ -40623,7 +40623,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1684" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1684" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1684" s="1">
         <v>1683</v>
       </c>
@@ -40643,7 +40643,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1685" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1685" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1685" s="1">
         <v>1684</v>
       </c>
@@ -40663,7 +40663,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1686" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1686" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1686" s="1">
         <v>1685</v>
       </c>
@@ -40683,7 +40683,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1687" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1687" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1687" s="1">
         <v>1686</v>
       </c>
@@ -40703,7 +40703,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1688" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1688" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1688" s="1">
         <v>1687</v>
       </c>
@@ -40723,7 +40723,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1689" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1689" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1689" s="1">
         <v>1688</v>
       </c>
@@ -40743,7 +40743,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1690" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1690" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1690" s="1">
         <v>1689</v>
       </c>
@@ -40763,7 +40763,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1691" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1691" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1691" s="1">
         <v>1690</v>
       </c>
@@ -40783,7 +40783,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1692" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1692" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1692" s="1">
         <v>1691</v>
       </c>
@@ -40803,7 +40803,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1693" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1693" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1693" s="1">
         <v>1692</v>
       </c>
@@ -40823,7 +40823,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1694" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1694" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1694" s="1">
         <v>1693</v>
       </c>
@@ -40843,7 +40843,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1695" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1695" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1695" s="1">
         <v>1694</v>
       </c>
@@ -40863,7 +40863,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1696" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1696" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1696" s="1">
         <v>1695</v>
       </c>
@@ -40883,7 +40883,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1697" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1697" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1697" s="1">
         <v>1696</v>
       </c>
@@ -40903,7 +40903,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1698" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1698" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1698" s="1">
         <v>1697</v>
       </c>
@@ -40923,7 +40923,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1699" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1699" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1699" s="1">
         <v>1698</v>
       </c>
@@ -40943,7 +40943,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1700" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1700" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1700" s="1">
         <v>1699</v>
       </c>
@@ -40963,7 +40963,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1701" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1701" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1701" s="1">
         <v>1700</v>
       </c>
@@ -40983,7 +40983,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1702" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1702" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1702" s="1">
         <v>1701</v>
       </c>
@@ -41003,7 +41003,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1703" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1703" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1703" s="1">
         <v>1702</v>
       </c>
@@ -41023,7 +41023,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1704" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1704" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1704" s="1">
         <v>1703</v>
       </c>
@@ -41043,7 +41043,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1705" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1705" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1705" s="1">
         <v>1704</v>
       </c>
@@ -41063,7 +41063,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1706" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1706" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1706" s="1">
         <v>1705</v>
       </c>
@@ -41083,7 +41083,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1707" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1707" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1707" s="1">
         <v>1706</v>
       </c>
@@ -41103,7 +41103,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1708" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1708" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1708" s="1">
         <v>1707</v>
       </c>
@@ -41123,7 +41123,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1709" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1709" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1709" s="1">
         <v>1708</v>
       </c>
@@ -41143,7 +41143,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1710" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1710" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1710" s="1">
         <v>1709</v>
       </c>
@@ -41163,7 +41163,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1711" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1711" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1711" s="1">
         <v>1710</v>
       </c>
@@ -41183,7 +41183,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1712" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1712" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1712" s="1">
         <v>1711</v>
       </c>
@@ -41203,7 +41203,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1713" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1713" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1713" s="1">
         <v>1712</v>
       </c>
@@ -41223,7 +41223,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1714" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1714" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1714" s="1">
         <v>1713</v>
       </c>
@@ -41243,7 +41243,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1715" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1715" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1715" s="1">
         <v>1714</v>
       </c>
@@ -41263,7 +41263,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1716" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1716" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1716" s="1">
         <v>1715</v>
       </c>
@@ -41283,7 +41283,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1717" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1717" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1717" s="1">
         <v>1716</v>
       </c>
@@ -41303,7 +41303,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1718" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1718" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1718" s="1">
         <v>1717</v>
       </c>
@@ -41323,7 +41323,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1719" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1719" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1719" s="1">
         <v>1718</v>
       </c>
@@ -41343,7 +41343,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1720" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1720" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1720" s="1">
         <v>1719</v>
       </c>
@@ -41363,7 +41363,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1721" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1721" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1721" s="1">
         <v>1720</v>
       </c>
@@ -41383,7 +41383,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1722" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1722" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1722" s="1">
         <v>1721</v>
       </c>
@@ -41403,7 +41403,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1723" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1723" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1723" s="1">
         <v>1722</v>
       </c>
@@ -41423,7 +41423,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1724" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1724" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1724" s="1">
         <v>1723</v>
       </c>
@@ -41443,7 +41443,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1725" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1725" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1725" s="1">
         <v>1724</v>
       </c>
@@ -41463,7 +41463,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1726" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1726" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1726" s="1">
         <v>1725</v>
       </c>
@@ -41483,7 +41483,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1727" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1727" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1727" s="1">
         <v>1726</v>
       </c>
@@ -41503,7 +41503,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1728" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1728" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1728" s="1">
         <v>1727</v>
       </c>
@@ -41523,7 +41523,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1729" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1729" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1729" s="1">
         <v>1728</v>
       </c>
@@ -41543,7 +41543,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1730" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1730" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1730" s="1">
         <v>1729</v>
       </c>
@@ -41563,7 +41563,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1731" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1731" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1731" s="1">
         <v>1730</v>
       </c>
@@ -41583,7 +41583,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1732" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1732" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1732" s="1">
         <v>1731</v>
       </c>
@@ -41603,7 +41603,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1733" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1733" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1733" s="1">
         <v>1732</v>
       </c>
@@ -41623,7 +41623,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1734" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1734" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1734" s="1">
         <v>1733</v>
       </c>
@@ -41643,7 +41643,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1735" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1735" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1735" s="1">
         <v>1734</v>
       </c>
@@ -41663,7 +41663,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1736" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1736" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1736" s="1">
         <v>1735</v>
       </c>
@@ -41683,7 +41683,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1737" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1737" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1737" s="1">
         <v>1736</v>
       </c>
@@ -41703,7 +41703,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1738" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1738" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1738" s="1">
         <v>1737</v>
       </c>
@@ -41723,7 +41723,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1739" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1739" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1739" s="1">
         <v>1738</v>
       </c>
@@ -41743,7 +41743,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1740" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1740" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1740" s="1">
         <v>1739</v>
       </c>
@@ -41763,7 +41763,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1741" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1741" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1741" s="1">
         <v>1740</v>
       </c>
@@ -41783,7 +41783,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1742" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1742" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1742" s="1">
         <v>1741</v>
       </c>
@@ -41803,7 +41803,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1743" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1743" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1743" s="1">
         <v>1742</v>
       </c>
@@ -41823,7 +41823,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1744" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1744" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1744" s="1">
         <v>1743</v>
       </c>
@@ -41843,7 +41843,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1745" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1745" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1745" s="1">
         <v>1744</v>
       </c>
@@ -41863,7 +41863,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1746" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1746" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1746" s="1">
         <v>1745</v>
       </c>
@@ -41883,7 +41883,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1747" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1747" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1747" s="1">
         <v>1746</v>
       </c>
@@ -41903,7 +41903,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1748" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1748" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1748" s="1">
         <v>1747</v>
       </c>
@@ -41923,7 +41923,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1749" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1749" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1749" s="1">
         <v>1748</v>
       </c>
@@ -41943,7 +41943,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1750" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1750" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1750" s="1">
         <v>1749</v>
       </c>
@@ -45743,21 +45743,21 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="1940" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1940" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A1940" s="1">
         <v>1939</v>
       </c>
       <c r="B1940" t="s">
-        <v>2019</v>
+        <v>2087</v>
       </c>
       <c r="C1940" t="s">
-        <v>847</v>
-      </c>
-      <c r="D1940" s="4" t="s">
-        <v>313</v>
-      </c>
-      <c r="E1940" s="4" t="s">
-        <v>678</v>
+        <v>530</v>
+      </c>
+      <c r="D1940" t="s">
+        <v>664</v>
+      </c>
+      <c r="E1940" t="s">
+        <v>665</v>
       </c>
       <c r="F1940" t="s">
         <v>2112</v>
@@ -48163,7 +48163,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2061" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2061" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2061" s="1">
         <v>2060</v>
       </c>
@@ -48183,7 +48183,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2062" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2062" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2062" s="1">
         <v>2061</v>
       </c>
@@ -48203,7 +48203,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2063" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2063" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2063" s="1">
         <v>2062</v>
       </c>
@@ -48223,7 +48223,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2064" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2064" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2064" s="1">
         <v>2063</v>
       </c>
@@ -48243,7 +48243,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2065" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2065" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2065" s="1">
         <v>2064</v>
       </c>
@@ -48263,7 +48263,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2066" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2066" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2066" s="1">
         <v>2065</v>
       </c>
@@ -48283,7 +48283,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2067" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2067" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2067" s="1">
         <v>2066</v>
       </c>
@@ -48303,7 +48303,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2068" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2068" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2068" s="1">
         <v>2067</v>
       </c>
@@ -48323,7 +48323,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2069" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2069" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2069" s="1">
         <v>2068</v>
       </c>
@@ -48343,7 +48343,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2070" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2070" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2070" s="1">
         <v>2069</v>
       </c>
@@ -48363,7 +48363,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2071" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2071" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2071" s="1">
         <v>2070</v>
       </c>
@@ -48383,7 +48383,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2072" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2072" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2072" s="1">
         <v>2071</v>
       </c>
@@ -48403,7 +48403,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2073" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2073" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2073" s="1">
         <v>2072</v>
       </c>
@@ -48423,7 +48423,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2074" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2074" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2074" s="1">
         <v>2073</v>
       </c>
@@ -48443,7 +48443,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2075" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2075" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2075" s="1">
         <v>2074</v>
       </c>
@@ -48463,7 +48463,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2076" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2076" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2076" s="1">
         <v>2075</v>
       </c>
@@ -48483,7 +48483,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2077" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2077" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2077" s="1">
         <v>2076</v>
       </c>
@@ -48503,7 +48503,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2078" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2078" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2078" s="1">
         <v>2077</v>
       </c>
@@ -48523,7 +48523,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2079" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2079" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2079" s="1">
         <v>2078</v>
       </c>
@@ -48543,7 +48543,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2080" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2080" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2080" s="1">
         <v>2079</v>
       </c>
@@ -48563,7 +48563,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2081" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2081" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2081" s="1">
         <v>2080</v>
       </c>
@@ -48583,7 +48583,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="2082" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2082" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2082" s="1">
         <v>2081</v>
       </c>
@@ -53608,16 +53608,16 @@
         <v>2332</v>
       </c>
       <c r="B2333" t="s">
-        <v>2021</v>
+        <v>2091</v>
       </c>
       <c r="C2333" t="s">
-        <v>1591</v>
+        <v>2093</v>
       </c>
       <c r="D2333" t="s">
-        <v>1639</v>
+        <v>664</v>
       </c>
       <c r="E2333" t="s">
-        <v>1640</v>
+        <v>665</v>
       </c>
       <c r="F2333" t="s">
         <v>2112</v>
@@ -56845,13 +56845,16 @@
     </row>
   </sheetData>
   <autoFilter ref="B1:F2494" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="2">
+    <filterColumn colId="0">
       <filters>
-        <filter val="total_assets"/>
+        <filter val="Detailed Ownership (Monthly)"/>
+        <filter val="Detailed Ownership with History (Monthly)"/>
+        <filter val="Key Ownership (Monthly)"/>
+        <filter val="Ownership History (Semi-Annual)"/>
       </filters>
     </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:F2494">
-      <sortCondition descending="1" ref="F1:F2494"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B41:F2333">
+      <sortCondition ref="D1:D2494"/>
     </sortState>
   </autoFilter>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>